<commit_message>
Vorlage-Blatt: erste Zeile als Beispielfall ausgefuellt
- Blatt 'Vorlage (leer)' -> 'Vorlage' mit einer Musterzeile (Strom-Fall MS12),
  zeigt gruene Sparte-Faerbung und die komplette Status-Ampel; als Beispiel
  markiert ('bitte ueberschreiben oder loeschen')

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DcPKW57M51qyYEs8uR4niV
</commit_message>
<xml_diff>
--- a/infra_Wohnanlagenverzeichnis_Vorlage.xlsx
+++ b/infra_Wohnanlagenverzeichnis_Vorlage.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="HV Baum" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Vorlage (leer)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vorlage" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Listen" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Hinweise" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -16,7 +16,7 @@
     <definedName name="ArtListe">Listen!$A$2:$A$4</definedName>
     <definedName name="SparteListe">Listen!$B$2:$B$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HV Baum'!$A$4:$R$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Vorlage (leer)'!$A$4:$R$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Vorlage'!$A$4:$R$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4305,24 +4305,94 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" s="10" t="n"/>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="10" t="n"/>
-      <c r="P5" s="10" t="n"/>
-      <c r="Q5" s="10" t="n"/>
-      <c r="R5" s="13" t="n"/>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>MS12</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Musterstraße 12</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>90402 Nürnberg</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>N-ERGIE</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>1EMH0010457812</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>85000</v>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Ja 01.01.2027</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>N-ERGIE</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>1105999001</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>Zustimmung</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>Zustimmung</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t>Beispielzeile – bitte überschreiben oder löschen</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="14" t="n"/>

</xml_diff>